<commit_message>
Pre Market Thu 2026-06-18
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-06-18.xlsx
+++ b/market-prep/Pre Market 2026-06-18.xlsx
@@ -459,12 +459,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7504,70</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3++</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -476,12 +476,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30063,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3++</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -493,12 +493,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2975,31</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3++</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -510,12 +510,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52114,87</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3++</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>24934,67</t>
+          <t>24948,90</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>24493,95</t>
+          <t>24312,16</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -578,12 +578,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1,16</t>
+          <t>1,15</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6++</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4363,36</t>
+          <t>4252,47</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>70,80</t>
+          <t>67,83</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,12 +629,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1796,52</t>
+          <t>1737,66</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6++</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>79,33</t>
+          <t>79,55</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,12 +663,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>65935,28</t>
+          <t>64446,04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6++</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1777,26</t>
+          <t>1749,00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>17,08</t>
+          <t>18,84</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3,23%</t>
+          <t>12,37%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>93,14</t>
+          <t>95,52</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7504,78</t>
+          <t>7420,10</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>

</xml_diff>